<commit_message>
fixed issue with lecturer-parser reading the first row
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arzbe\IdeaProjects\TimetablePlanner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2248ED0A-02C3-40CB-8525-890F4E9A2DA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A78F79F-A359-4CB0-9866-E32454C41471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="1" xr2:uid="{EC82FCA3-5B96-47D8-BD7E-1C3F50D7DE8B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{EC82FCA3-5B96-47D8-BD7E-1C3F50D7DE8B}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t>Steven Hawkins</t>
   </si>
@@ -62,6 +62,21 @@
   </si>
   <si>
     <t>Alan Turing</t>
+  </si>
+  <si>
+    <t>Momo Lustig</t>
+  </si>
+  <si>
+    <t>Martin Lustiger</t>
+  </si>
+  <si>
+    <t>Anna Couch</t>
+  </si>
+  <si>
+    <t>Marilyn Monroe</t>
+  </si>
+  <si>
+    <t>Frank Sinatra</t>
   </si>
 </sst>
 </file>
@@ -433,12 +448,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DAD1A16-556F-4F10-8A98-B67B873665B7}">
   <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" customWidth="1"/>
+    <col min="1" max="1" width="17.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -455,12 +470,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26F7DCC9-4F44-465E-BF30-CAC24A6588F8}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.140625" customWidth="1"/>
+    <col min="1" max="1" width="22.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -468,7 +483,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -479,12 +494,12 @@
         <v>44808</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -492,7 +507,7 @@
         <v>44814</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -500,7 +515,7 @@
         <v>44813</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -512,9 +527,43 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B8AB866-154E-4DEA-A187-603755020D91}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <dimension ref="A1:A6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>